<commit_message>
Map Hardest difficulty to Extreme
Just Dance 4 and 2014 called the top difficulty tier "Hardest"; from
Just Dance 2015 on the same tier is "Extreme" (the wiki lists e.g. Good
Feeling and Blurred Lines Extreme Versions as Hardest in their original
game and Extreme in Unlimited). Relabels the 10 JD4/JD2014 Extreme
Versions so difficulty uses only Easy/Medium/Hard/Extreme, and
regenerates songlist.xlsx to match.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Prvp2CYZoRF45PL5zfmtrB
</commit_message>
<xml_diff>
--- a/songlist.xlsx
+++ b/songlist.xlsx
@@ -54156,7 +54156,7 @@
       </c>
       <c r="I1661" t="inlineStr">
         <is>
-          <t>Hardest</t>
+          <t>Extreme</t>
         </is>
       </c>
     </row>
@@ -54620,7 +54620,7 @@
       </c>
       <c r="I1681" t="inlineStr">
         <is>
-          <t>Hardest</t>
+          <t>Extreme</t>
         </is>
       </c>
     </row>
@@ -55018,7 +55018,7 @@
       </c>
       <c r="I1698" t="inlineStr">
         <is>
-          <t>Hardest</t>
+          <t>Extreme</t>
         </is>
       </c>
     </row>
@@ -55540,7 +55540,7 @@
       </c>
       <c r="I1721" t="inlineStr">
         <is>
-          <t>Hardest</t>
+          <t>Extreme</t>
         </is>
       </c>
     </row>
@@ -55992,7 +55992,7 @@
       </c>
       <c r="I1739" t="inlineStr">
         <is>
-          <t>Hardest</t>
+          <t>Extreme</t>
         </is>
       </c>
     </row>
@@ -56148,7 +56148,7 @@
       </c>
       <c r="I1745" t="inlineStr">
         <is>
-          <t>Hardest</t>
+          <t>Extreme</t>
         </is>
       </c>
     </row>
@@ -56304,7 +56304,7 @@
       </c>
       <c r="I1751" t="inlineStr">
         <is>
-          <t>Hardest</t>
+          <t>Extreme</t>
         </is>
       </c>
     </row>
@@ -56482,7 +56482,7 @@
       </c>
       <c r="I1758" t="inlineStr">
         <is>
-          <t>Hardest</t>
+          <t>Extreme</t>
         </is>
       </c>
     </row>
@@ -56578,7 +56578,7 @@
       </c>
       <c r="I1762" t="inlineStr">
         <is>
-          <t>Hardest</t>
+          <t>Extreme</t>
         </is>
       </c>
     </row>
@@ -56652,7 +56652,7 @@
       </c>
       <c r="I1765" t="inlineStr">
         <is>
-          <t>Hardest</t>
+          <t>Extreme</t>
         </is>
       </c>
     </row>

</xml_diff>